<commit_message>
Cap nhat bai tho moi: 26/06/2026 14:01
</commit_message>
<xml_diff>
--- a/Tho_chiet_ly_cuoc_song_FullVersion.xlsx
+++ b/Tho_chiet_ly_cuoc_song_FullVersion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\THO VE CUOC SONG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0428801B-A5EF-405C-85B1-4A48DFB8FE0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0890A1CA-F462-421E-AEDC-1AA24B5D0768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Danh Sách Bài Thơ" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="724">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="730">
   <si>
     <t>STT</t>
   </si>
@@ -2887,12 +2887,54 @@
   <si>
     <t>→ Danh Sách (hàng 66)</t>
   </si>
+  <si>
+    <t>HÀO KHÍ PHỤC HƯNG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Phục Hưng một dải niềm tin
+Vươn lên từ những công trình dựng xây
+Bao năm dãi nắng dầm mây
+Giữ trọn chữ tín tháng ngày chẳng phai
+Khắp miền Bắc, Trung, Nam dài
+Dấu chân người thợ miệt mài sớm trưa
+Dựng cao mái ấm bao mùa
+Góp xây đất nước như xưa hẹn lòng
+Đoàn kết một dạ một lòng
+Vượt bao thử thách, qua vòng gian nan
+Khát vọng còn mãi ngút ngàn
+Phục Hưng vững bước, vẻ vang tháng ngày
+Chuyển mình theo nhịp thời gian
+AI cùng dữ liệu mở ngàn đường đi
+Công trường kết nối tức thì
+Phục Hưng vững bước, chẳng vì gian nan
+BIM lưu trữ muôn vàn
+Tiến độ, chất lượng rõ ràng từng phân
+Dashboard quản trị chuyên cần
+Giúp cho quyết sách thêm phần vững tin
+Kỷ cương làm gốc trường sinh
+Sáng tạo làm cánh hành trình vươn xa
+Chung tay dựng nghiệp Sơn Hà
+Phục Hưng giàu mạnh, sáng lòa tương lai.</t>
+  </si>
+  <si>
+    <t>📖 Mở bài 67</t>
+  </si>
+  <si>
+    <t>→ Danh Sách (hàng 67)</t>
+  </si>
+  <si>
+    <t>Khơi dạy</t>
+  </si>
+  <si>
+    <t>khơi dạy hào khí</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2912,11 +2954,13 @@
       <sz val="14"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -2933,6 +2977,7 @@
     <font>
       <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -2955,46 +3000,68 @@
       <sz val="13"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF1F4E79"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF1F4E79"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF595959"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="9"/>
       <color rgb="FF0563C1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="14">
@@ -3113,10 +3180,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3238,8 +3306,15 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -3540,7 +3615,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr defaultColWidth="18" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.28515625" bestFit="1" customWidth="1"/>
@@ -4871,7 +4946,36 @@
         <v>264</v>
       </c>
     </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" s="5">
+        <v>66</v>
+      </c>
+      <c r="B67" s="18" t="s">
+        <v>724</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>728</v>
+      </c>
+      <c r="D67" s="6">
+        <v>15</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>729</v>
+      </c>
+      <c r="F67" s="46" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" s="5"/>
+      <c r="B68" s="6"/>
+      <c r="C68" s="6"/>
+      <c r="D68" s="6"/>
+      <c r="E68" s="6"/>
+      <c r="F68" s="11"/>
+    </row>
   </sheetData>
+  <phoneticPr fontId="19" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="F2" location="'Nội Dung Bài Thơ'!A3" display="📖 Mở bài 1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="F3" location="'Nội Dung Bài Thơ'!A4" display="📖 Mở bài 2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
@@ -4938,6 +5042,7 @@
     <hyperlink ref="F64" location="'Nội Dung Bài Thơ'!A65" display="📖 Mở bài 63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
     <hyperlink ref="F65" location="'Nội Dung Bài Thơ'!A66" display="📖 Mở bài 64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
     <hyperlink ref="F66" location="'Nội Dung Bài Thơ'!A67" display="📖 Mở bài 65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="F67" location="'Nội Dung Bài Thơ'!A68" display="📖 Mở bài 67" xr:uid="{96C309DB-024F-4F4D-A34F-193F77CEB720}"/>
   </hyperlinks>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0"/>
@@ -6155,7 +6260,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -7294,6 +7399,23 @@
       </c>
       <c r="E67" s="21" t="s">
         <v>723</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="360" x14ac:dyDescent="0.25">
+      <c r="A68" s="17">
+        <v>66</v>
+      </c>
+      <c r="B68" s="18" t="s">
+        <v>724</v>
+      </c>
+      <c r="C68" s="19" t="s">
+        <v>725</v>
+      </c>
+      <c r="D68" s="20" t="s">
+        <v>722</v>
+      </c>
+      <c r="E68" s="45" t="s">
+        <v>727</v>
       </c>
     </row>
   </sheetData>
@@ -7366,6 +7488,7 @@
     <hyperlink ref="E65" location="'Danh Sách Bài Thơ'!A64" display="→ Danh Sách (hàng 64)" xr:uid="{00000000-0004-0000-0300-00003E000000}"/>
     <hyperlink ref="E66" location="'Danh Sách Bài Thơ'!A65" display="→ Danh Sách (hàng 65)" xr:uid="{00000000-0004-0000-0300-00003F000000}"/>
     <hyperlink ref="E67" location="'Danh Sách Bài Thơ'!A66" display="→ Danh Sách (hàng 66)" xr:uid="{00000000-0004-0000-0300-000040000000}"/>
+    <hyperlink ref="E68" location="'Danh Sách Bài Thơ'!A67" display="→ Danh Sách (hàng 67)" xr:uid="{E6825638-B004-494C-B4C2-427E16FC12DC}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Tich hop module hoc tieng trung va cap nhat service worker v2
</commit_message>
<xml_diff>
--- a/Tho_chiet_ly_cuoc_song_FullVersion.xlsx
+++ b/Tho_chiet_ly_cuoc_song_FullVersion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\THO VE CUOC SONG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0890A1CA-F462-421E-AEDC-1AA24B5D0768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C01922D5-AEE5-47E7-B060-215AF0F8B854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3290,6 +3290,12 @@
     <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3304,12 +3310,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4962,7 +4962,7 @@
       <c r="E67" s="6" t="s">
         <v>729</v>
       </c>
-      <c r="F67" s="46" t="s">
+      <c r="F67" s="38" t="s">
         <v>726</v>
       </c>
     </row>
@@ -5065,14 +5065,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="42" t="s">
         <v>265</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
     </row>
     <row r="2" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
@@ -5098,7 +5098,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="37" t="s">
+      <c r="A3" s="39" t="s">
         <v>273</v>
       </c>
       <c r="B3" s="7" t="s">
@@ -5121,7 +5121,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="38"/>
+      <c r="A4" s="40"/>
       <c r="B4" s="7" t="s">
         <v>280</v>
       </c>
@@ -5142,7 +5142,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="38"/>
+      <c r="A5" s="40"/>
       <c r="B5" s="7" t="s">
         <v>286</v>
       </c>
@@ -5163,7 +5163,7 @@
       </c>
     </row>
     <row r="6" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="38"/>
+      <c r="A6" s="40"/>
       <c r="B6" s="7" t="s">
         <v>292</v>
       </c>
@@ -5184,7 +5184,7 @@
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="38"/>
+      <c r="A7" s="40"/>
       <c r="B7" s="7" t="s">
         <v>298</v>
       </c>
@@ -5205,7 +5205,7 @@
       </c>
     </row>
     <row r="8" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="38"/>
+      <c r="A8" s="40"/>
       <c r="B8" s="7" t="s">
         <v>304</v>
       </c>
@@ -5226,7 +5226,7 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="39"/>
+      <c r="A9" s="41"/>
       <c r="B9" s="7" t="s">
         <v>309</v>
       </c>
@@ -5247,7 +5247,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="37" t="s">
+      <c r="A10" s="39" t="s">
         <v>315</v>
       </c>
       <c r="B10" s="7" t="s">
@@ -5270,7 +5270,7 @@
       </c>
     </row>
     <row r="11" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="38"/>
+      <c r="A11" s="40"/>
       <c r="B11" s="7" t="s">
         <v>321</v>
       </c>
@@ -5291,7 +5291,7 @@
       </c>
     </row>
     <row r="12" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="38"/>
+      <c r="A12" s="40"/>
       <c r="B12" s="7" t="s">
         <v>327</v>
       </c>
@@ -5312,7 +5312,7 @@
       </c>
     </row>
     <row r="13" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="38"/>
+      <c r="A13" s="40"/>
       <c r="B13" s="7" t="s">
         <v>333</v>
       </c>
@@ -5333,7 +5333,7 @@
       </c>
     </row>
     <row r="14" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="38"/>
+      <c r="A14" s="40"/>
       <c r="B14" s="7" t="s">
         <v>338</v>
       </c>
@@ -5354,7 +5354,7 @@
       </c>
     </row>
     <row r="15" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="38"/>
+      <c r="A15" s="40"/>
       <c r="B15" s="7" t="s">
         <v>344</v>
       </c>
@@ -5375,7 +5375,7 @@
       </c>
     </row>
     <row r="16" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="39"/>
+      <c r="A16" s="41"/>
       <c r="B16" s="7" t="s">
         <v>350</v>
       </c>
@@ -5396,7 +5396,7 @@
       </c>
     </row>
     <row r="17" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="37" t="s">
+      <c r="A17" s="39" t="s">
         <v>355</v>
       </c>
       <c r="B17" s="7" t="s">
@@ -5419,7 +5419,7 @@
       </c>
     </row>
     <row r="18" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="38"/>
+      <c r="A18" s="40"/>
       <c r="B18" s="7" t="s">
         <v>362</v>
       </c>
@@ -5440,7 +5440,7 @@
       </c>
     </row>
     <row r="19" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="38"/>
+      <c r="A19" s="40"/>
       <c r="B19" s="7" t="s">
         <v>366</v>
       </c>
@@ -5461,7 +5461,7 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="38"/>
+      <c r="A20" s="40"/>
       <c r="B20" s="7" t="s">
         <v>372</v>
       </c>
@@ -5482,7 +5482,7 @@
       </c>
     </row>
     <row r="21" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="38"/>
+      <c r="A21" s="40"/>
       <c r="B21" s="7" t="s">
         <v>378</v>
       </c>
@@ -5503,7 +5503,7 @@
       </c>
     </row>
     <row r="22" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="38"/>
+      <c r="A22" s="40"/>
       <c r="B22" s="7" t="s">
         <v>383</v>
       </c>
@@ -5524,7 +5524,7 @@
       </c>
     </row>
     <row r="23" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="38"/>
+      <c r="A23" s="40"/>
       <c r="B23" s="7" t="s">
         <v>389</v>
       </c>
@@ -5545,7 +5545,7 @@
       </c>
     </row>
     <row r="24" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="39"/>
+      <c r="A24" s="41"/>
       <c r="B24" s="7" t="s">
         <v>395</v>
       </c>
@@ -5566,7 +5566,7 @@
       </c>
     </row>
     <row r="25" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="37" t="s">
+      <c r="A25" s="39" t="s">
         <v>401</v>
       </c>
       <c r="B25" s="7" t="s">
@@ -5589,7 +5589,7 @@
       </c>
     </row>
     <row r="26" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="38"/>
+      <c r="A26" s="40"/>
       <c r="B26" s="7" t="s">
         <v>407</v>
       </c>
@@ -5610,7 +5610,7 @@
       </c>
     </row>
     <row r="27" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="38"/>
+      <c r="A27" s="40"/>
       <c r="B27" s="7" t="s">
         <v>413</v>
       </c>
@@ -5631,7 +5631,7 @@
       </c>
     </row>
     <row r="28" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="38"/>
+      <c r="A28" s="40"/>
       <c r="B28" s="7" t="s">
         <v>419</v>
       </c>
@@ -5652,7 +5652,7 @@
       </c>
     </row>
     <row r="29" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="38"/>
+      <c r="A29" s="40"/>
       <c r="B29" s="7" t="s">
         <v>424</v>
       </c>
@@ -5673,7 +5673,7 @@
       </c>
     </row>
     <row r="30" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="38"/>
+      <c r="A30" s="40"/>
       <c r="B30" s="7" t="s">
         <v>429</v>
       </c>
@@ -5694,7 +5694,7 @@
       </c>
     </row>
     <row r="31" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="38"/>
+      <c r="A31" s="40"/>
       <c r="B31" s="7" t="s">
         <v>434</v>
       </c>
@@ -5715,7 +5715,7 @@
       </c>
     </row>
     <row r="32" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="38"/>
+      <c r="A32" s="40"/>
       <c r="B32" s="7" t="s">
         <v>440</v>
       </c>
@@ -5736,7 +5736,7 @@
       </c>
     </row>
     <row r="33" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="38"/>
+      <c r="A33" s="40"/>
       <c r="B33" s="7" t="s">
         <v>446</v>
       </c>
@@ -5757,7 +5757,7 @@
       </c>
     </row>
     <row r="34" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="38"/>
+      <c r="A34" s="40"/>
       <c r="B34" s="7" t="s">
         <v>450</v>
       </c>
@@ -5778,7 +5778,7 @@
       </c>
     </row>
     <row r="35" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="39"/>
+      <c r="A35" s="41"/>
       <c r="B35" s="7" t="s">
         <v>455</v>
       </c>
@@ -5860,12 +5860,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="44" t="s">
         <v>461</v>
       </c>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
@@ -6271,13 +6271,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="46" t="s">
         <v>522</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
     </row>
     <row r="2" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
@@ -7231,7 +7231,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" ht="192" x14ac:dyDescent="0.25">
       <c r="A58" s="22">
         <v>56</v>
       </c>
@@ -7414,7 +7414,7 @@
       <c r="D68" s="20" t="s">
         <v>722</v>
       </c>
-      <c r="E68" s="45" t="s">
+      <c r="E68" s="37" t="s">
         <v>727</v>
       </c>
     </row>

</xml_diff>